<commit_message>
add tugas 1 : import file (level, user, kategori, supplier)
</commit_message>
<xml_diff>
--- a/PWLPOS/public/template_barang.xlsx
+++ b/PWLPOS/public/template_barang.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\WebLanjut\PWLPOS\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F54E1E1-8BB3-46CC-A640-2FC9987197A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F119F3FB-47DD-46FD-B987-1DF79378A5F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10245" yWindow="0" windowWidth="10245" windowHeight="10920" xr2:uid="{C73FB3FA-5830-4131-BD46-4804A4229B17}"/>
+    <workbookView xWindow="1275" yWindow="780" windowWidth="8865" windowHeight="7995" xr2:uid="{C73FB3FA-5830-4131-BD46-4804A4229B17}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>kategori_id</t>
   </si>
@@ -36,40 +36,70 @@
     <t>harga_jual</t>
   </si>
   <si>
-    <t>SBK-003</t>
-  </si>
-  <si>
-    <t>SNK-003</t>
-  </si>
-  <si>
-    <t>MND-003</t>
-  </si>
-  <si>
-    <t>BAY-003</t>
-  </si>
-  <si>
-    <t>MNM-003</t>
-  </si>
-  <si>
-    <t>Telur Omega (10 butir)</t>
-  </si>
-  <si>
-    <t>Sari Roti</t>
-  </si>
-  <si>
-    <t>Shampo Pantene</t>
-  </si>
-  <si>
-    <t>Baju Bayi 2th</t>
-  </si>
-  <si>
-    <t>Cleo 600ml</t>
-  </si>
-  <si>
     <t>kode_barang</t>
   </si>
   <si>
     <t>nama_barang</t>
+  </si>
+  <si>
+    <t>SB001</t>
+  </si>
+  <si>
+    <t>Sabun Cuci</t>
+  </si>
+  <si>
+    <t>PN001</t>
+  </si>
+  <si>
+    <t>Pensil</t>
+  </si>
+  <si>
+    <t>MG001</t>
+  </si>
+  <si>
+    <t>Mug</t>
+  </si>
+  <si>
+    <t>PL001</t>
+  </si>
+  <si>
+    <t>Pulpen</t>
+  </si>
+  <si>
+    <t>GK001</t>
+  </si>
+  <si>
+    <t>Gantungan Kunci</t>
+  </si>
+  <si>
+    <t>BK001</t>
+  </si>
+  <si>
+    <t>Buku Tulis</t>
+  </si>
+  <si>
+    <t>TL001</t>
+  </si>
+  <si>
+    <t>Tali Rafia</t>
+  </si>
+  <si>
+    <t>KP001</t>
+  </si>
+  <si>
+    <t>Karpet</t>
+  </si>
+  <si>
+    <t>LM001</t>
+  </si>
+  <si>
+    <t>Lampu Meja</t>
+  </si>
+  <si>
+    <t>SP001</t>
+  </si>
+  <si>
+    <t>Sepeda</t>
   </si>
 </sst>
 </file>
@@ -113,9 +143,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -430,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE7719F3-BEC1-4478-83E1-16B94E1ED57E}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -445,10 +480,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
@@ -458,88 +493,173 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2">
+        <v>5000</v>
+      </c>
+      <c r="E2" s="2">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E3" s="2">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2">
-        <v>22000</v>
-      </c>
-      <c r="E2">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2">
+        <v>7000</v>
+      </c>
+      <c r="E4" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2">
+        <v>2000</v>
+      </c>
+      <c r="E5" s="2">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3">
-        <v>11500</v>
-      </c>
-      <c r="E3">
-        <v>12500</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="2">
+        <v>3000</v>
+      </c>
+      <c r="E6" s="2">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>2</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="2">
+        <v>4000</v>
+      </c>
+      <c r="E7" s="2">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="2">
+        <v>2500</v>
+      </c>
+      <c r="E8" s="2">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4">
-        <v>17500</v>
-      </c>
-      <c r="E4">
-        <v>18500</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="B9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2">
+        <v>50000</v>
+      </c>
+      <c r="E9" s="2">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>3</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="2">
+        <v>15000</v>
+      </c>
+      <c r="E10" s="2">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
         <v>6</v>
       </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5">
-        <v>89000</v>
-      </c>
-      <c r="E5">
-        <v>92500</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6">
-        <v>3750</v>
-      </c>
-      <c r="E6">
-        <v>4300</v>
+      <c r="B11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="2">
+        <v>500000</v>
+      </c>
+      <c r="E11" s="2">
+        <v>900000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>